<commit_message>
Taco Shop Business Plan Kit F2: ensamblado, gates G1-G9 y revisión adversarial (0 B · 5 M · 8 m, todo arreglado, cifras sin mover)
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/taco-shop-business-plan/taco-cost-trompo-yield-calculator.xlsx
+++ b/astro-site/public/dl/taco-shop-business-plan/taco-cost-trompo-yield-calculator.xlsx
@@ -1487,7 +1487,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>B. HOMEMADE (masa harina, tortilla machine and a tortillera)</t>
+          <t>B. HOMEMADE (masa harina, tortilla machine and a tortilla maker)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1564,7 +1564,7 @@
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Yearly cost of a tortillera ($, with payroll costs)</t>
+          <t>Yearly cost of the tortilla maker ($, with payroll costs)</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
@@ -3805,7 +3805,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>1. Type the price of the case, the tortillas per case and the weight of each tortilla, plus the masa harina, machine and tortillera numbers. The tortillas per lb bought are what you need to order from your supplier.</t>
+          <t>1. Type the price of the case, the tortillas per case and the weight of each tortilla, plus the masa harina, machine and tortilla maker numbers. The tortillas per lb bought are what you need to order from your supplier.</t>
         </is>
       </c>
     </row>

</xml_diff>